<commit_message>
Complete PCW metadata for configured samples
</commit_message>
<xml_diff>
--- a/metadata/samples_meta.xlsx
+++ b/metadata/samples_meta.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10322"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10810"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/alyssaflint/Documents/Research/Luo - PhD/FC Xenium/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45A4EFD5-D6D4-8D41-B821-D1F889EBEAB0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8986DCFC-AFA3-9948-8B1F-F9BF0EF58AC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-22880" yWindow="4560" windowWidth="12320" windowHeight="9980" xr2:uid="{E563D142-85BA-4E30-940A-4620E61C5369}"/>
+    <workbookView xWindow="-24700" yWindow="1500" windowWidth="24220" windowHeight="18460" xr2:uid="{E563D142-85BA-4E30-940A-4620E61C5369}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="23">
   <si>
     <t>sample</t>
   </si>
@@ -96,6 +96,15 @@
   </si>
   <si>
     <t>FB124_X_G</t>
+  </si>
+  <si>
+    <t>GZFB_20_X_G</t>
+  </si>
+  <si>
+    <t>GZFB_22_X_G</t>
+  </si>
+  <si>
+    <t>PCW19</t>
   </si>
 </sst>
 </file>
@@ -467,7 +476,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{19CA858D-9EB6-40C3-8A97-6805BE2A3E6C}">
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B13"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="11.6640625" bestFit="1" customWidth="1"/>
@@ -561,6 +570,22 @@
         <v>6</v>
       </c>
     </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>20</v>
+      </c>
+      <c r="B12" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>21</v>
+      </c>
+      <c r="B13" t="s">
+        <v>22</v>
+      </c>
+    </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A1:B11">
     <sortCondition ref="B1:B11"/>

</xml_diff>